<commit_message>
feat: sync accounts and categories from web and redesign template to accounting ledger
- Add metadata_fetcher to extract active accounts (excluding strike-through) and income/expense categories from dailyexpenses4.com.
- Redesign Excel and CSV templates to Accounting Ledger layout with separate Expense and Income columns.
- Implement conditional Excel DataValidation for Category (Income categories if Income column is set, Expense categories if Expense column is set).
- Support transfer transactions via Expense column and 'Source -> Target' account syntax.
- Add -s / --sync-metadata CLI command and --sync flag to template generator.
- Add unit tests for metadata caching and generic CSV ledger parsing.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -482,19 +482,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D34"/>
+  <dimension ref="B2:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>🏦 Daily Expenses 4 Importer — Setup &amp; Accounts</t>
+          <t>🏦 Daily Expenses 4 Importer — Setup &amp; Categories</t>
         </is>
       </c>
     </row>
@@ -508,240 +510,273 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>1. Write your exact Daily Expenses 4 Account names in Column B (e.g. 'Checking Account', 'Credit Card', 'Cash').</t>
+          <t>1. Column B lists your active Accounts (synced from your Daily Expenses 4 app).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2. Review or customize your Categories in Column D.</t>
+          <t>2. Column D lists your Expense Categories; Column F lists your Income Categories.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>3. Go to the 'Movements' sheet and enter your transactions using the dropdown lists.</t>
+          <t>3. Go to the 'Movements' sheet and enter transactions in Accounting Ledger format (Expense vs Income).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>4. In the 'Date &amp; Time' column, use YYYY-MM-DD HH:MM:SS format (e.g. 2026-09-15 14:30:00).</t>
+          <t>4. When you enter an amount in 'Income', the Category dropdown automatically shows Income categories!</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>5. To import, run: daily-expenses-importer -i template.xlsx</t>
+          <t>5. For transfers, enter the amount in 'Expense' and use 'Source -&gt; Target' in the 'Account' column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>6. In 'Date &amp; Time', use YYYY-MM-DD HH:MM:SS format (e.g. 2026-09-15 14:30:00).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>7. To import, run: daily-expenses-importer -i template.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Accounts</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Categories</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Checking Account</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Bills</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Credit Card</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Clothing</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Expense Categories</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Income Categories</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>BanPa Personal</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Autopista</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Pago préstamos</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Savings</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Bebidas</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Préstamo</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Entertainment</t>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
         </is>
       </c>
     </row>
     <row r="16">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Fuel</t>
+          <t>Diversión</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Ventas</t>
         </is>
       </c>
     </row>
     <row r="17">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Euros</t>
+        </is>
+      </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Groceries</t>
+          <t>Educación</t>
         </is>
       </c>
     </row>
     <row r="18">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>TDC - Banesco</t>
+        </is>
+      </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Gasolina</t>
         </is>
       </c>
     </row>
     <row r="19">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>USD - Cash</t>
+        </is>
+      </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Hijo</t>
         </is>
       </c>
     </row>
     <row r="20">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Zinli</t>
+        </is>
+      </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Hogar</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Hotel</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Kids</t>
+          <t>Mascota</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Merchandise</t>
+          <t>Mercancía</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Negocio</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Otros</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Pets</t>
+          <t>Personales</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Subscriptions</t>
+          <t>Propinas</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Tips</t>
+          <t>Préstamo</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Toll</t>
+          <t>Restaurante</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Transfer</t>
+          <t>Ropa</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Salud</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Tecnología</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Utilities</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Vehicle</t>
+          <t>Transporte</t>
         </is>
       </c>
     </row>
@@ -761,9 +796,9 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -780,17 +815,17 @@
       </c>
       <c r="C1" s="6" t="inlineStr">
         <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
           <t>Category</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>Type</t>
         </is>
       </c>
       <c r="F1" s="6" t="inlineStr">
@@ -810,22 +845,18 @@
           <t>Supermarket Groceries</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Groceries</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="n">
+      <c r="C2" s="7" t="n">
         <v>45.5</v>
       </c>
+      <c r="D2" s="5" t="n"/>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Autopista</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Checking Account</t>
+          <t>BanPa Personal</t>
         </is>
       </c>
     </row>
@@ -840,22 +871,18 @@
           <t>Monthly Salary Deposit</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Income</t>
-        </is>
-      </c>
+      <c r="C3" s="5" t="n"/>
       <c r="D3" s="7" t="n">
         <v>1500</v>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Pago préstamos</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Checking Account</t>
+          <t>BanPa Personal</t>
         </is>
       </c>
     </row>
@@ -870,22 +897,14 @@
           <t>Credit Card Payment</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Transfer</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="n">
+      <c r="C4" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Transfer</t>
-        </is>
-      </c>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Checking Account -&gt; Credit Card</t>
+          <t>BanPa Personal -&gt; Binance</t>
         </is>
       </c>
     </row>
@@ -900,22 +919,18 @@
           <t>Pharmacy &amp; Medicine</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n">
+      <c r="C5" s="7" t="n">
         <v>12.3</v>
       </c>
+      <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Bebidas</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Checking Account</t>
+          <t>BanPa Personal</t>
         </is>
       </c>
     </row>
@@ -930,35 +945,28 @@
           <t>Restaurant Dinner</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Dining</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="n">
+      <c r="C6" s="7" t="n">
         <v>34</v>
       </c>
+      <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Autopista</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Binance</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Type" error="Select a valid movement type (Expense, Income, Transfer)" type="list">
-      <formula1>"Expense,Income,Transfer"</formula1>
+  <dataValidations count="2">
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Category" error="Select a category from the list or configure it in the Setup sheet" type="list">
+      <formula1>=IF(ISNUMBER($D2), Setup!$F$13:$F$16, Setup!$D$13:$D$33)</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Category" error="Select a category from the list or add it in the Setup sheet" type="list">
-      <formula1>=Setup!$D$11:$D$40</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Account" error="Select an account from the list or add it in the Setup sheet" type="list">
-      <formula1>=Setup!$B$11:$B$30</formula1>
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Account" error="Select an account from the list or configure it in the Setup sheet" type="list">
+      <formula1>=Setup!$B$13:$B$20</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>